<commit_message>
Map replication outputs to source code
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -89,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -99,6 +99,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,79 +436,1236 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D78"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="58" customWidth="1"/>
+    <col min="2" max="2" width="70" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>2</v>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data Preparation Program</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dataset created</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Line Number</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reproduced?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/01_antenna_tower_griddist_mapping.R</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/02_gen_tower_maghrib_and_sunset_time.py</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/03_gen_compressed_panel.py</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/04_gen_outage_ind.py</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/05_gen_towerday_indicators_panel.py</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/06_gen_hash_towerday_panel.py</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/07_panel_gridmonth_or_districtmonth.py</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/08_01_gen_hash_homelocations.py</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/08_02_gen_hash_districtmonth_continuity_ind.py</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/08_03_panel_gridmonth_or_districtmonth_restricted.py</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/09_01_gen_hash_level_relig.py</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/09_02_gen_init_hash_relig.py</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/09_03_gen_hashqtr_panel.py</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/10_SIGACTS_merge_cdr.R</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/11_01_220805_create_master.do</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/11_02_220824_create_master_shortcode.do</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/11_03_250108_update_master_cdr.do</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/12_240213_gen_widewheat_panel.do</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/13_precleaning_alltables.do</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cdr_and_conflict_dm.dta</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">266</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/13_precleaning_alltables.do</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cdr_and_climate_gm.dta</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">530</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/13_precleaning_alltables.do</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cdr_and_climate_gy.dta</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">639</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/13_precleaning_alltables.do</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">calls_shortcode_comparison_dm.dta</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">677</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/13_precleaning_alltables.do</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">calls_shortcode_comparison_gm.dta</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">706</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/13_precleaning_alltables.do</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dist_level.dta</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">910</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/13_precleaning_alltables.do</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid_level.dta</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">922</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure/Table #</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Program</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Line Number</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reproduced?</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure 1</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/Fig1.R</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="34" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure 2</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/Fig2.R</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">114, 246</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="34" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure 3</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/Fig3.R</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">119</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure 4</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/Fig4.R</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">150</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure A1</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No program provided</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identified</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure A2</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/FigA2.qmd</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">84 (synthetic tower data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="34" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure A3</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/FigA3.R</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">75</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure A4</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/FigA4.R</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70-72</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure A5</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/FigA5.R</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">219-223, 231-235</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="34" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figure A6</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/FigA6.R</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">125</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="34" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table 1</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">145</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="34" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table 2</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="34" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table 3</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">291</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="34" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A1</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">333</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A2</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">432, 441, 448, 454, 460, 466, 472 (synthetic data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="34" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A3</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">508 (synthetic data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="34" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A4</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">555</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="34" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A5</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">629, 642, 650, 661</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="34" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A6</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">749, 761, 779, 796, 809, 823, 830</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="34" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A7</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">859</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="34" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A8</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">940</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="34" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A9</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">996</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="34" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A10</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1062</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="34" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A11</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1115</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="34" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A12</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1162</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="34" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A13</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/TabA13.R</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">465 (synthetic data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="34" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table A14</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15" customHeight="1"/>
+    <row r="57" ht="24" customHeight="1">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In-text numbers</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Program</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Line Number</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reproduced?</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="52" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF pp. 1-2: roughly 23 billion calls; over 10 million unique users and 22.6 billion calls.</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No code identified; relevant raw-data cleaning programs are NUL-only</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="52" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 3: a one-SD survey religiosity increase is associated with a 27% increase in the Maghrib dip. Later text and Table A2 report 29%.</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No code generates the 27% claim</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="52" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 10: 90% of Afghans are Sunni; prayer starts within 15 minutes; Shia Maghrib begins 5-15 minutes later; Zuhr/Asr last three hours and Maghrib less than one hour.</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No package program; institutional background</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="52" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 11: U.S. church attendance over-reporting ranges from 100% to over 400%; Afghan adult mobile-phone penetration is 60%-70%.</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No package program; externally cited background</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="52" customHeight="1">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 12: 6.0-7.7 million numbers per year, population 39 million, and 22.6 billion calls.</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No code identified; relevant raw-data cleaning programs are NUL-only</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="52" customHeight="1">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 12: 1,739 towers across 292 of 398 districts and subscriber/population correlation rho = 0.94.</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/FigA2.qmd</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71 comments only on 1,739 towers; no calculation for the remaining claims</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="52" customHeight="1">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 13 n. 17: tower-month quartile dips of 13%, 21%, 27%, and 36%.</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/Fig1.R</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not identifiable: file contains only NUL bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="52" customHeight="1">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 21: 72% of subscribers make a shortcode call; shortcode calls are 3% of total call volume.</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No code identified</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="52" customHeight="1">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 21 n. 23: adult literacy rate is 43%.</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No package program; externally cited background</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="52" customHeight="1">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 21 n. 24: SMS locations are interpolated within the same hour (16%), day (47%), or month (37%).</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No reviewable code; relevant cleaning programs are NUL-only</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="52" customHeight="1">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 21 n. 25: 43% of data transactions occur within 5 seconds and 47% within one minute.</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No reviewable code; relevant cleaning programs are NUL-only</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="52" customHeight="1">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF pp. 22-23: survey has 1,090 people and six practices; the stated 48-month CDR period conflicts with Jan. 2015-Dec. 2016 (24 months); median use is three calls/day. Table A6 reports 1,092 observations.</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No code generates these claims; Table A6 is written by Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">823 (Table A6 output)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="52" customHeight="1">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 24 n. 30: survey composition is 71% Tajik, 17% Pashtun, 9% Hazara, and 3% other.</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No code or exhibit reports the full composition</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="52" customHeight="1">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 29: SIGACTS locations have five-decimal/one-meter precision and the overlapping sample contains 95,231 incidents.</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/FigA5.R</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">75-108 filters/processes events but does not report these quantities</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="52" customHeight="1">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 30: incident-category totals are 27,931; 57,629; 4,285; and 27,155.</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/FigA5.R</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="52" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 34 n. 41: results are unchanged using 1% or 10% Hazara-share thresholds.</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/All_Tables.do</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">970, 1010 implement only the 5% threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="52" customHeight="1">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 36: agriculture is 23% of GDP and supplies income to 62% of the population.</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No package program; externally cited background</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="52" customHeight="1">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 36 n. 43: temperature rose 1.8 C since 1950; crop areas are 2.3, 0.33, 0.27, 0.22, 0.15, and 0.12 million hectares.</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No package program; externally cited background</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="52" customHeight="1">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 40 n. 49: approximately 19% of grid cells are urban.</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/13_precleaning_alltables.do</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">408 defines the urban indicator but does not calculate 19%</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="52" customHeight="1">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF pp. 44-45: individual-quarter analysis uses approximately 8.5 million subscribers and a 33-month 2013-2015 baseline.</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Analysis/TabA13.R</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">437 states 33 months; no code reports the 8.5 million count</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="52" customHeight="1">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper PDF p. 48 n. 58: almost 41% of poppy-cultivation observations are missing.</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code/Cleaning/13_precleaning_alltables.do</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">110-125 create missing-value indicators but do not calculate 41%</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>